<commit_message>
Daily NSE scan: 2026-08-28
</commit_message>
<xml_diff>
--- a/output/2026-08-28/enriched_analysis.xlsx
+++ b/output/2026-08-28/enriched_analysis.xlsx
@@ -1900,27 +1900,27 @@
         <v>331.05</v>
       </c>
       <c r="J15" t="n">
-        <v>311.69</v>
+        <v>314.32</v>
       </c>
       <c r="K15" t="n">
-        <v>6.2</v>
+        <v>5.3</v>
       </c>
       <c r="L15" t="n">
         <v>63.24</v>
       </c>
       <c r="M15" t="n">
-        <v>1.41</v>
+        <v>1.74</v>
       </c>
       <c r="N15" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>31-07-2026</t>
+          <t>28-08-2026</t>
         </is>
       </c>
       <c r="P15" t="n">
-        <v>0.446</v>
+        <v>0.551</v>
       </c>
       <c r="Q15" t="n">
         <v>316</v>
@@ -5679,23 +5679,23 @@
         <v>331.05</v>
       </c>
       <c r="D15" t="n">
-        <v>311.69</v>
+        <v>314.32</v>
       </c>
       <c r="E15" t="n">
-        <v>6.2</v>
+        <v>5.3</v>
       </c>
       <c r="F15" t="n">
         <v>63.24</v>
       </c>
       <c r="G15" t="n">
-        <v>1.41</v>
+        <v>1.74</v>
       </c>
       <c r="H15" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>31-07-2026</t>
+          <t>28-08-2026</t>
         </is>
       </c>
     </row>

</xml_diff>